<commit_message>
added bfs and dfs
</commit_message>
<xml_diff>
--- a/graphs.xlsx
+++ b/graphs.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\GECBH\AAD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23D6312F-C73F-4460-A7D4-8D7186033B89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43F570F0-1E0A-4DA9-8B60-16C21953C70A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{E1285DE0-0D4D-4DB6-BFD0-649F41EFE9C6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{E1285DE0-0D4D-4DB6-BFD0-649F41EFE9C6}"/>
   </bookViews>
   <sheets>
     <sheet name="bubbleSort" sheetId="1" r:id="rId1"/>
-    <sheet name="search" sheetId="2" r:id="rId2"/>
+    <sheet name="merge sort" sheetId="3" r:id="rId2"/>
+    <sheet name="bfs" sheetId="4" r:id="rId3"/>
+    <sheet name="dfs" sheetId="5" r:id="rId4"/>
+    <sheet name="search" sheetId="2" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="9">
   <si>
     <t>Size</t>
   </si>
@@ -56,15 +59,28 @@
   <si>
     <t>Binary Search time (s)</t>
   </si>
+  <si>
+    <t>Merge Sort(s)</t>
+  </si>
+  <si>
+    <t>Selection Sort(s)</t>
+  </si>
+  <si>
+    <t>No of Vertices</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Execution time (s) </t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.000000"/>
+    <numFmt numFmtId="165" formatCode="0.00000000"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -78,6 +94,31 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -87,7 +128,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -110,11 +151,63 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -123,11 +216,31 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -181,8 +294,13 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-GB"/>
-              <a:t>Comparison of Bubble Sort and Quick Sort</a:t>
+              <a:t>Bubble Sort VS</a:t>
             </a:r>
+            <a:r>
+              <a:rPr lang="en-GB" baseline="0"/>
+              <a:t> Quick Sort</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-GB"/>
           </a:p>
         </c:rich>
       </c:tx>
@@ -211,7 +329,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-US"/>
+          <a:endParaRPr lang="en-GB"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -219,7 +337,7 @@
     <c:plotArea>
       <c:layout/>
       <c:scatterChart>
-        <c:scatterStyle val="lineMarker"/>
+        <c:scatterStyle val="smoothMarker"/>
         <c:varyColors val="0"/>
         <c:ser>
           <c:idx val="0"/>
@@ -290,27 +408,27 @@
                 <c:formatCode>0.000000</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>0.26300000000000001</c:v>
+                  <c:v>0.29099999999999998</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>7.3559999999999999</c:v>
+                  <c:v>8.7330000000000005</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>30.95</c:v>
+                  <c:v>32.854999999999997</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>127.172</c:v>
+                  <c:v>126.97799999999999</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>301.04899999999998</c:v>
+                  <c:v>281.95999999999998</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
-          <c:smooth val="0"/>
+          <c:smooth val="1"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-B8EA-4C39-8101-1CE0A4E5BE0D}"/>
+              <c16:uniqueId val="{00000000-1B71-418A-A561-172B32095271}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -386,24 +504,24 @@
                   <c:v>1E-3</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>6.0000000000000001E-3</c:v>
+                  <c:v>7.0000000000000001E-3</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.2999999999999999E-2</c:v>
+                  <c:v>1.6E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2.7E-2</c:v>
+                  <c:v>3.5999999999999997E-2</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>6.0999999999999999E-2</c:v>
+                  <c:v>4.7E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
-          <c:smooth val="0"/>
+          <c:smooth val="1"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-B8EA-4C39-8101-1CE0A4E5BE0D}"/>
+              <c16:uniqueId val="{00000001-1B71-418A-A561-172B32095271}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -415,11 +533,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="1135468352"/>
-        <c:axId val="1960068176"/>
+        <c:axId val="1253598192"/>
+        <c:axId val="1163170479"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="1135468352"/>
+        <c:axId val="1253598192"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -460,8 +578,13 @@
                 </a:pPr>
                 <a:r>
                   <a:rPr lang="en-GB"/>
-                  <a:t>Array Size (n)</a:t>
+                  <a:t>No. of</a:t>
                 </a:r>
+                <a:r>
+                  <a:rPr lang="en-GB" baseline="0"/>
+                  <a:t> elements</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-GB"/>
               </a:p>
             </c:rich>
           </c:tx>
@@ -490,7 +613,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-US"/>
+              <a:endParaRPr lang="en-GB"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -531,12 +654,12 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1960068176"/>
+        <c:crossAx val="1163170479"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="1960068176"/>
+        <c:axId val="1163170479"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -577,7 +700,11 @@
                 </a:pPr>
                 <a:r>
                   <a:rPr lang="en-GB"/>
-                  <a:t>Execution Time (seconds)</a:t>
+                  <a:t>Time</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-GB" baseline="0"/>
+                  <a:t> for execution</a:t>
                 </a:r>
               </a:p>
             </c:rich>
@@ -648,7 +775,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1135468352"/>
+        <c:crossAx val="1253598192"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -769,6 +896,631 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
+              <a:rPr lang="en-GB"/>
+              <a:t>Merge Sort</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-GB" baseline="0"/>
+              <a:t> vs Selection Sort</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-GB"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-GB"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="smoothMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'merge sort'!$B$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Merge Sort(s)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'merge sort'!$A$2:$A$8</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2000</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>5000</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>7000</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>10000</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>50000</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>500000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'merge sort'!$B$2:$B$8</c:f>
+              <c:numCache>
+                <c:formatCode>0.000000</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>9.9999999999999995E-7</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3.0000000000000001E-6</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3.0000000000000001E-6</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1E-3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1E-3</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>7.0000000000000001E-3</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.108</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-3D73-41C8-A9C0-67E24270FA9D}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'merge sort'!$C$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Selection Sort(s)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'merge sort'!$A$2:$A$8</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2000</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>5000</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>7000</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>10000</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>50000</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>500000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'merge sort'!$C$2:$C$8</c:f>
+              <c:numCache>
+                <c:formatCode>0.000000</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>2E-3</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>6.0000000000000001E-3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>5.6000000000000001E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>8.7999999999999995E-2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.14199999999999999</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>4.0970000000000004</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>340.68299999999999</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-3D73-41C8-A9C0-67E24270FA9D}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1253654800"/>
+        <c:axId val="1163172879"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1253654800"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-GB" sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:sysClr val="windowText" lastClr="000000">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:sysClr>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t>No. of elements</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1163172879"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1163172879"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-GB"/>
+                  <a:t>Time of execution</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="0.000000" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1253654800"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-GB"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
               <a:rPr lang="en-GB" sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
                 <a:solidFill>
                   <a:sysClr val="windowText" lastClr="000000">
@@ -886,25 +1638,25 @@
             <c:numRef>
               <c:f>search!$B$2:$B$7</c:f>
               <c:numCache>
-                <c:formatCode>0.000000</c:formatCode>
+                <c:formatCode>0.00000000</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>2E-3</c:v>
+                  <c:v>0.05</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>6.4000000000000001E-2</c:v>
+                  <c:v>0.13900000000000001</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.126</c:v>
+                  <c:v>0.16300000000000001</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.63500000000000001</c:v>
+                  <c:v>0.84699999999999998</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>6.3890000000000002</c:v>
+                  <c:v>6.4269999999999996</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>13.026</c:v>
+                  <c:v>13.146000000000001</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -983,27 +1735,24 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>search!$C$2:$C$7</c:f>
+              <c:f>search!$C$2:$C$6</c:f>
               <c:numCache>
-                <c:formatCode>0.000000</c:formatCode>
-                <c:ptCount val="6"/>
+                <c:formatCode>0.00000000</c:formatCode>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>1.9999999999999999E-6</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>0.01</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>2E-3</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>3.0000000000000001E-3</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>4.0000000000000001E-3</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1220,11 +1969,11 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-US"/>
+              <a:endParaRPr lang="en-GB"/>
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="0.000000" sourceLinked="1"/>
+        <c:numFmt formatCode="0.00000000" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1262,6 +2011,622 @@
           </a:p>
         </c:txPr>
         <c:crossAx val="1784302224"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-GB"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-GB"/>
+              <a:t> LINEAR</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-GB" baseline="0"/>
+              <a:t> VS BINARY SEARCH</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-GB"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-GB"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="smoothMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>search!$B$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v> Linear Search time (s)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>search!$A$2:$A$7</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>10000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>50000</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>100000</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>500000</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5000000</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>10000000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>search!$B$2:$B$7</c:f>
+              <c:numCache>
+                <c:formatCode>0.00000000</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>0.05</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.13900000000000001</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.16300000000000001</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.84699999999999998</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>6.4269999999999996</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>13.146000000000001</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-0871-4AA9-914B-19E120B96F2B}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>search!$C$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Binary Search time (s)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>search!$A$2:$A$7</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>10000</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>50000</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>100000</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>500000</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5000000</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>10000000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>search!$C$2:$C$7</c:f>
+              <c:numCache>
+                <c:formatCode>0.00000000</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>1.9999999999999999E-6</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.01</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2E-3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3.0000000000000001E-3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4.0000000000000001E-3</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5.0000000000000001E-3</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-0871-4AA9-914B-19E120B96F2B}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1273732064"/>
+        <c:axId val="1163136399"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1273732064"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-GB"/>
+                  <a:t>Size</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-GB" baseline="0"/>
+                  <a:t> of array</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-GB"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-GB"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1163136399"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1163136399"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-GB"/>
+                  <a:t>Time</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-GB" baseline="0"/>
+                  <a:t> taken for execution</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-GB"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-GB"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="0.00000000" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1273732064"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1428,6 +2793,86 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
@@ -2460,27 +3905,1059 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>514350</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>90487</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>252412</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>42862</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>209550</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>166687</xdr:rowOff>
+      <xdr:colOff>557212</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>119062</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="3" name="Chart 2">
+        <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DBAD9085-2989-9AA3-78B1-9CDAFD627244}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{324BF51E-1A99-A2F9-E6BA-C62C39FA31A4}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2502,6 +4979,47 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>585787</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>52387</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>280987</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>128587</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6E879A13-26AB-5E27-473C-4452B330DE37}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
@@ -2534,6 +5052,42 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>476250</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>90487</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>171450</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>166687</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2AD553BB-CD4F-ABAF-DC6F-4704F126FEE9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2882,7 +5436,7 @@
         <v>10000</v>
       </c>
       <c r="B2" s="3">
-        <v>0.26300000000000001</v>
+        <v>0.29099999999999998</v>
       </c>
       <c r="C2" s="3">
         <v>1E-3</v>
@@ -2893,10 +5447,10 @@
         <v>50000</v>
       </c>
       <c r="B3" s="3">
-        <v>7.3559999999999999</v>
+        <v>8.7330000000000005</v>
       </c>
       <c r="C3" s="3">
-        <v>6.0000000000000001E-3</v>
+        <v>7.0000000000000001E-3</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -2904,10 +5458,10 @@
         <v>100000</v>
       </c>
       <c r="B4" s="3">
-        <v>30.95</v>
+        <v>32.854999999999997</v>
       </c>
       <c r="C4" s="3">
-        <v>1.2999999999999999E-2</v>
+        <v>1.6E-2</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -2915,10 +5469,10 @@
         <v>200000</v>
       </c>
       <c r="B5" s="3">
-        <v>127.172</v>
+        <v>126.97799999999999</v>
       </c>
       <c r="C5" s="3">
-        <v>2.7E-2</v>
+        <v>3.5999999999999997E-2</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -2926,10 +5480,10 @@
         <v>300000</v>
       </c>
       <c r="B6" s="3">
-        <v>301.04899999999998</v>
+        <v>281.95999999999998</v>
       </c>
       <c r="C6" s="3">
-        <v>6.0999999999999999E-2</v>
+        <v>4.7E-2</v>
       </c>
     </row>
   </sheetData>
@@ -2939,89 +5493,332 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78BE6867-564C-490C-927E-AF743B55C0AD}">
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="16.5703125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="20.28515625" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="4">
+        <v>1000</v>
+      </c>
+      <c r="B2" s="10">
+        <v>9.9999999999999995E-7</v>
+      </c>
+      <c r="C2" s="10">
+        <v>2E-3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="2">
+        <v>2000</v>
+      </c>
+      <c r="B3" s="10">
+        <v>3.0000000000000001E-6</v>
+      </c>
+      <c r="C3" s="10">
+        <v>6.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
+        <v>5000</v>
+      </c>
+      <c r="B4" s="10">
+        <v>3.0000000000000001E-6</v>
+      </c>
+      <c r="C4" s="10">
+        <v>5.6000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="2">
+        <v>7000</v>
+      </c>
+      <c r="B5" s="10">
+        <v>1E-3</v>
+      </c>
+      <c r="C5" s="10">
+        <v>8.7999999999999995E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="2">
+        <v>10000</v>
+      </c>
+      <c r="B6" s="10">
+        <v>1E-3</v>
+      </c>
+      <c r="C6" s="10">
+        <v>0.14199999999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="2">
+        <v>50000</v>
+      </c>
+      <c r="B7" s="10">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="C7" s="10">
+        <v>4.0970000000000004</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
+        <v>500000</v>
+      </c>
+      <c r="B8" s="10">
+        <v>0.108</v>
+      </c>
+      <c r="C8" s="10">
+        <v>340.68299999999999</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CDBA7272-86AF-4F6C-BB1E-48449703CA96}">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="2" max="2" width="28.28515625" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="12">
+        <v>10</v>
+      </c>
+      <c r="B2" s="14">
+        <v>1E-3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="12">
+        <v>100</v>
+      </c>
+      <c r="B3" s="14">
+        <v>1E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="12">
+        <v>500</v>
+      </c>
+      <c r="B4" s="14">
+        <v>2E-3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="12">
+        <v>3892</v>
+      </c>
+      <c r="B5" s="14">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="12">
+        <v>7057</v>
+      </c>
+      <c r="B6" s="14">
+        <v>0.17199999999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="12">
+        <v>50515</v>
+      </c>
+      <c r="B7" s="14">
+        <v>25.055</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E2C81A3-470C-4061-B3DB-4CE2DEBE2917}">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="25.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="15">
+        <v>10</v>
+      </c>
+      <c r="B2" s="16">
+        <v>1E-3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="16">
+        <v>100</v>
+      </c>
+      <c r="B3" s="16">
+        <v>6.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="16">
+        <v>475</v>
+      </c>
+      <c r="B4" s="16">
+        <v>7.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="16">
+        <v>7115</v>
+      </c>
+      <c r="B5" s="16">
+        <v>0.156</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="16">
+        <v>10876</v>
+      </c>
+      <c r="B6" s="16">
+        <v>0.313</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="17">
+        <v>75879</v>
+      </c>
+      <c r="B7" s="16">
+        <v>31.552</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F140C91-F1F4-4530-B43A-5F83BDD03F9F}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="21" style="1" customWidth="1"/>
-    <col min="3" max="3" width="22.5703125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="21" style="6" customWidth="1"/>
+    <col min="3" max="3" width="22.5703125" style="6" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="7" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="7">
+      <c r="A2" s="8">
         <v>10000</v>
       </c>
-      <c r="B2" s="6">
-        <v>2E-3</v>
-      </c>
-      <c r="C2" s="6">
-        <v>0</v>
+      <c r="B2" s="9">
+        <v>0.05</v>
+      </c>
+      <c r="C2" s="9">
+        <v>1.9999999999999999E-6</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="7">
+      <c r="A3" s="8">
         <v>50000</v>
       </c>
-      <c r="B3" s="6">
-        <v>6.4000000000000001E-2</v>
-      </c>
-      <c r="C3" s="6">
-        <v>0</v>
+      <c r="B3" s="9">
+        <v>0.13900000000000001</v>
+      </c>
+      <c r="C3" s="9">
+        <v>0.01</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="7">
+      <c r="A4" s="8">
         <v>100000</v>
       </c>
-      <c r="B4" s="6">
-        <v>0.126</v>
-      </c>
-      <c r="C4" s="6">
-        <v>0</v>
+      <c r="B4" s="9">
+        <v>0.16300000000000001</v>
+      </c>
+      <c r="C4" s="9">
+        <v>2E-3</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="7">
+      <c r="A5" s="8">
         <v>500000</v>
       </c>
-      <c r="B5" s="6">
-        <v>0.63500000000000001</v>
-      </c>
-      <c r="C5" s="6">
-        <v>0</v>
+      <c r="B5" s="9">
+        <v>0.84699999999999998</v>
+      </c>
+      <c r="C5" s="9">
+        <v>3.0000000000000001E-3</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="7">
+      <c r="A6" s="8">
         <v>5000000</v>
       </c>
-      <c r="B6" s="6">
-        <v>6.3890000000000002</v>
-      </c>
-      <c r="C6" s="6">
-        <v>0</v>
+      <c r="B6" s="9">
+        <v>6.4269999999999996</v>
+      </c>
+      <c r="C6" s="9">
+        <v>4.0000000000000001E-3</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="7">
+      <c r="A7" s="8">
         <v>10000000</v>
       </c>
-      <c r="B7" s="6">
-        <v>13.026</v>
-      </c>
-      <c r="C7" s="6">
-        <v>0</v>
+      <c r="B7" s="9">
+        <v>13.146000000000001</v>
+      </c>
+      <c r="C7" s="9">
+        <v>5.0000000000000001E-3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>